<commit_message>
feat(jobs): add WordPress-powered job board foundation
</commit_message>
<xml_diff>
--- a/docs/Apex_HR_Master_Sitemap_and_URL_Register.xlsx
+++ b/docs/Apex_HR_Master_Sitemap_and_URL_Register.xlsx
@@ -1111,10 +1111,10 @@
         <x:v>/jobs/</x:v>
       </x:c>
       <x:c r="F12" s="46" t="str">
-        <x:v>Provisional</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="G12" s="37" t="str">
-        <x:v>Pending gate</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H12" s="37" t="str">
         <x:v>P2</x:v>
@@ -1124,7 +1124,7 @@
         <x:v>Functional Requirements Document</x:v>
       </x:c>
       <x:c r="K12" s="37" t="str">
-        <x:v>Archive route recognised; ATS source pending</x:v>
+        <x:v>Public Job Board powered by the WordPress vacancy feed; canonical Next.js route</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1142,10 +1142,10 @@
         <x:v>/jobs/[job-slug]/</x:v>
       </x:c>
       <x:c r="F13" s="46" t="str">
-        <x:v>Provisional</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="G13" s="37" t="str">
-        <x:v>Pending gate</x:v>
+        <x:v>Open vacancies only</x:v>
       </x:c>
       <x:c r="H13" s="37" t="str">
         <x:v>P2</x:v>
@@ -1155,7 +1155,7 @@
         <x:v>Functional Requirements Document</x:v>
       </x:c>
       <x:c r="K13" s="37" t="str">
-        <x:v>Dynamic pattern; only live approved vacancies index</x:v>
+        <x:v>Only published, open, non-expired roles are indexable; WordPress front end and sitemaps disabled</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -40449,6 +40449,29 @@
         <x:v>Use existing Contact enquiry flow; do not introduce unapproved commercial terms.</x:v>
       </x:c>
     </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="38" t="str">
+        <x:v>D-019</x:v>
+      </x:c>
+      <x:c r="B18" s="38" t="str">
+        <x:v>WordPress-powered Job Board</x:v>
+      </x:c>
+      <x:c r="C18" s="38" t="str">
+        <x:v>Confirm /jobs/ as the public Job Board and WordPress as vacancy source until ATS selection; only published, open, non-expired vacancies indexable.</x:v>
+      </x:c>
+      <x:c r="D18" s="38" t="str">
+        <x:v>Resolved</x:v>
+      </x:c>
+      <x:c r="E18" s="38" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="F18" s="38" t="str">
+        <x:v>WordPress vacancy CPT, Next.js routes and vacancy sitemap</x:v>
+      </x:c>
+      <x:c r="G18" s="38" t="str">
+        <x:v>WordPress vacancy pages and sitemaps disabled; applications and private CVs remain in Supabase.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>

</xml_diff>